<commit_message>
refactor: restructure project with OOP and add Chat with PDF feature
- Split monolithic main.py into modular OOP architecture
- core/pdf_processor.py: PDFProcessor + PDFDocument dataclass
- core/ai_engine.py: AIEngine with summarize + chat + retry logic
- ui/theme.py: ThemeManager singleton with Observer pattern
- ui/sidebar.py: Sidebar widget with StatCards
- ui/chat_panel.py: Chat UI with message bubbles
- app.py: main controller connecting all components
- main.py: entry point (5 lines)
</commit_message>
<xml_diff>
--- a/extracted_data.xlsx
+++ b/extracted_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,113 +479,6 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PI Docs</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>How to prompt engineer
-All prompting techniques — from clarity and examples to XML structuring, role
-prompting, thinking, and prompt chaining — are covered in Prompting best practices.
-That's the living reference; start there.
-The Claude Console also offers prompting tools—prompt generator, templates and
-variables, and prompt improver—to help you build and refine prompts quickly.
-Prompt engineering tutorial
-If you're an interactive learner, you can dive into our interactive tutorials instead!
-GitHub prompting tutorial
-An example-filled tutorial that covers the prompt engineering concepts found in our docs.
-Google Sheets prompting tutorial
-A lighter weight version of our prompt engineering tutorial via an interactive spreadsheet.
-Was this page helpful?</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Ask Docs</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Solutions Learn
-AI agents Blog</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Code modernization Catalog
-Coding Courses
-Customer support Use cases
-Education Connectors
-Financial services Customer stories
-Government Engineering at Anthropic
-Life sciences Events
-Powered by Claude
-Partners
-Service partners
-Amazon Bedrock Startups program
-Google Cloud's Vertex AI
-Company
-Anthropic
-Careers
-Economic Futures
-Research
-News
-Responsible Scaling Policy
-Security and compliance
-Transparency
-Help and security
-Availability
-Status
-Support
-Discord
-Terms and policies
-Privacy policy
-Responsible disclosure policy
-Terms of service: Commercial
-Terms of service: Consumer
-Usage policy
-Ask Docs</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>